<commit_message>
Update transfer record Excel with 23 entries
Co-authored-by: zhangliminabc <zhangliminabc@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/转账记录表.xlsx
+++ b/转账记录表.xlsx
@@ -439,15 +439,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,396 +457,608 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>银行卡号</t>
+          <t>卡号</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>日期</t>
+          <t>时间</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>时间</t>
+          <t>对方账号</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>银行</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>金额(元)</t>
+          <t>金额</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>代进</t>
+          <t>李锋</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>6217714807680485</t>
+          <t>6228411984527509979</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 18:52:17</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>19:51:31</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>中信银行</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>3888</v>
+          <t>6228411984527509979</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>3000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>刘美琳</t>
+          <t>艾赛提江·阿不多海提</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>6228482129185734774</t>
+          <t>6230520890070796273</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 18:57:17</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>19:55:10</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>农业银行</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>1300</v>
+          <t>6230520890070796273</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>郭佳慧</t>
+          <t>巩宪铎</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>6228481680593055716</t>
+          <t>6214830189072225</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 18:59:53</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>21:06:51</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>农业银行</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>3141</v>
+          <t>6214830189072225</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>1000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>王秀东</t>
+          <t>何锦</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>6228270407008347073</t>
+          <t>6230763000001198005</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 19:08:16</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>21:15:58</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>农业银行</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
-        <v>3000</v>
+          <t>6230763000001198005</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>4000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>屠文强</t>
+          <t>刘星臣</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>6213363469946407674</t>
+          <t>6228481257104701672</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 19:21:59</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>22:55:45</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>农业银行</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>1000</v>
+          <t>6228481257104701672</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>王曲格</t>
+          <t>阿尔满·斯拉木</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>6228230969012564976</t>
+          <t>6213363009980922673</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 19:34:13</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>23:00:10</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>农业银行</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>2200</v>
+          <t>6213363009980922673</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1500</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>韩德旺</t>
+          <t>欧述辛</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>6217890100003961468</t>
+          <t>6217995820005332418</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 19:36:12</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>23:09:55</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>中国银行</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>10000</v>
+          <t>6217995820005332418</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>郑汉明</t>
+          <t>林文强</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>6217281382000021929</t>
+          <t>6228480687106643475</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 19:38:12</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>23:12:55</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>广东省农村信用社联合社</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr"/>
+          <t>6228480687106643475</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>2800</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>杜富湘</t>
+          <t>尤康乐</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>6215826100000445807</t>
+          <t>6214835726776675</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 19:41:59</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>23:16:49</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>邮政储蓄银行</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>5890</v>
+          <t>6214835726776675</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>4500</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>王春林</t>
+          <t>买芳杰</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>6228480389549502075</t>
+          <t>6210812500002874283</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 19:44:35</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>23:19:12</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>农业银行</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>2200</v>
+          <t>6210812500002874283</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>1300</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>三义妞</t>
+          <t>田陆千</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>6214180002047673487</t>
+          <t>6216918801601725</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-29 19:47:05</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>23:22:17</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>宁波银行</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n">
-        <v>500</v>
+          <t>6216918801601725</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t>代进</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>6217714807680485</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 19:51:31</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>6217714807680485</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>3888</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>刘美琳</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>6228482129185734774</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 19:55:10</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>6228482129185734774</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>郭佳慧</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>6228481680593055716</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 21:06:51</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>6228481680593055716</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>3141</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>王秀东</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>6228270407008347073</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 21:15:58</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>6228270407008347073</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>屠文强</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>6213363469946407674</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 22:55:45</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>6213363469946407674</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>王曲格</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>6228230969012564976</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 23:00:10</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>6228230969012564976</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>韩德旺</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>6217890100003961468</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 23:09:55</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>6217890100003961468</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>郑汉明</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>6217281382000021929</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 23:12:55</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>6217281382000021929</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>杜富湘</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>6215826100000445807</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 23:16:49</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>6215826100000445807</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>5890</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>王春林</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>6228480389549502075</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 23:19:12</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>6228480389549502075</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>三义妞</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>6214180002047673487</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 23:22:17</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>6214180002047673487</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>王运峰</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>6217003860008425199</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>23:25:59</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>建设银行</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="n">
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29 23:25:59</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>6217003860008425199</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
         <v>8109</v>
       </c>
     </row>
-    <row r="15">
-      <c r="E15" s="3" t="inlineStr">
+    <row r="26">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="F15" s="3" t="n">
-        <v>41228</v>
+      <c r="E26" s="3" t="n">
+        <v>69828</v>
       </c>
     </row>
   </sheetData>

</xml_diff>